<commit_message>
Clinics call list: mobile numbers only (86)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/templates/קליניקות לייזר לשיחות.xlsx
+++ b/automation-agency/templates/קליניקות לייזר לשיחות.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תסריט" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'קליניקות'!$A$1:$K$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'קליניקות'!$A$1:$K$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -577,38 +577,42 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>א</t>
+          <t>ב</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>אליעד לוי - מרכז קוסמטי</t>
+          <t>נאווה דוק קוסמטיקה</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>אופקים</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>02-6240098</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr"/>
+          <t>050-8784997</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>וואטסאפ</t>
+        </is>
+      </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>85 ביקורות, ממוצע 5 · 85 ביקורות · דירוג 5</t>
+          <t>קוסמטיקה</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>ראיתי שיש לכן 85 ביקורות בדפי זהב, כלומר הרבה לקוחות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך באופקים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
@@ -624,38 +628,42 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>א</t>
+          <t>ב</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>מכון אחווה - חגית</t>
+          <t>בוהדנה הסרת שיער</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>אשקלון</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>02-6236036</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr"/>
+          <t>052-8101122</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>וואטסאפ</t>
+        </is>
+      </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>נוסד לפני 34 שנה על ידי חגית · 34 ביקורות · דירוג 4.6</t>
+          <t>הסרת שיער</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>ראיתי שיש לכן 34 ביקורות בדפי זהב, כלומר הרבה לקוחות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
@@ -671,38 +679,38 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>א</t>
+          <t>ב</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>מספרת שמפו</t>
+          <t>מאיה קליניק</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>אשקלון</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>דרום</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>02-6257666</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>20 שנה, טיפולי יופי ושיער במקום אחד · 11 ביקורות · דירוג 4.3</t>
-        </is>
-      </c>
+          <t>050-5858130</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>וואטסאפ</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr"/>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>ראיתי שיש לכן 11 ביקורות בדפי זהב, כלומר הרבה לקוחות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
@@ -723,12 +731,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>נאווה דוק קוסמטיקה</t>
+          <t>אלמה הסרת שיער</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>אופקים</t>
+          <t>אשקלון</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -738,7 +746,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>050-8784997</t>
+          <t>052-9555973</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -746,14 +754,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>קוסמטיקה</t>
-        </is>
-      </c>
+      <c r="H5" s="7" t="inlineStr"/>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך באופקים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
@@ -774,7 +778,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>בוהדנה הסרת שיער</t>
+          <t>ליאת קליניק</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -789,7 +793,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>052-8101122</t>
+          <t>050-6542911</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -797,11 +801,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער</t>
-        </is>
-      </c>
+      <c r="H6" s="7" t="inlineStr"/>
       <c r="I6" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -825,7 +825,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>מאיה קליניק</t>
+          <t>מהודרת</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>050-5858130</t>
+          <t>052-2341000</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>אלמה הסרת שיער</t>
+          <t>ילנה מור פתרונות אסתטיקה</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>052-9555973</t>
+          <t>054-5218052</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>ליאת קליניק</t>
+          <t>רפאל סופר הסרת שיער</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>050-6542911</t>
+          <t>058-6688148</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>מהודרת</t>
+          <t>אדרי שרון - הסרת שיער</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>אשקלון</t>
+          <t>באר שבע</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>052-2341000</t>
+          <t>050-4200002</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -989,10 +989,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער</t>
+        </is>
+      </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבאר שבע. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -1013,12 +1017,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>ילנה מור פתרונות אסתטיקה</t>
+          <t>Huda Laser Clinic</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>אשקלון</t>
+          <t>באר שבע</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1028,7 +1032,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>054-5218052</t>
+          <t>052-8687709</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1039,7 +1043,7 @@
       <c r="H11" s="7" t="inlineStr"/>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבאר שבע. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -1060,12 +1064,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>רפאל סופר הסרת שיער</t>
+          <t>איריס הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>אשקלון</t>
+          <t>דימונה</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1075,7 +1079,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>058-6688148</t>
+          <t>054-7702189</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -1083,10 +1087,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער בלייזר</t>
+        </is>
+      </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך באשקלון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בדימונה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -1107,12 +1115,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>אדרי שרון - הסרת שיער</t>
+          <t>מירי נעים</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>באר שבע</t>
+          <t>דימונה</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1122,7 +1130,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>050-4200002</t>
+          <t>050-4418442</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1130,14 +1138,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער</t>
-        </is>
-      </c>
+      <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבאר שבע. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בדימונה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -1158,12 +1162,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Huda Laser Clinic</t>
+          <t>חורי קליניקת לייזר</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>באר שבע</t>
+          <t>נתיבות</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1173,7 +1177,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>052-8687709</t>
+          <t>054-2529119</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1181,10 +1185,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>קליניקת לייזר</t>
+        </is>
+      </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבאר שבע. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בנתיבות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -1205,12 +1213,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>איריס הסרת שיער בלייזר</t>
+          <t>VS LASER &amp; BEAUTY</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>דימונה</t>
+          <t>נתיבות</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1220,7 +1228,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>054-7702189</t>
+          <t>053-5457519</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1228,14 +1236,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער בלייזר</t>
-        </is>
-      </c>
+      <c r="H15" s="7" t="inlineStr"/>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בדימונה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בנתיבות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -1256,12 +1260,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>מירי נעים</t>
+          <t>סנדרה קליניק</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>דימונה</t>
+          <t>ספיר</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1271,7 +1275,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>050-4418442</t>
+          <t>050-6594249</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1282,7 +1286,7 @@
       <c r="H16" s="7" t="inlineStr"/>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בדימונה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בספיר. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -1303,12 +1307,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>חורי קליניקת לייזר</t>
+          <t>חורי הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>נתיבות</t>
+          <t>ערד</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1318,7 +1322,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>054-2529119</t>
+          <t>050-9039052</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1326,14 +1330,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>קליניקת לייזר</t>
-        </is>
-      </c>
+      <c r="H17" s="7" t="inlineStr"/>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בנתיבות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בערד. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -1354,12 +1354,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>VS LASER &amp; BEAUTY</t>
+          <t>פלאש לייזר Flash Laser</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>נתיבות</t>
+          <t>קרית גת</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>053-5457519</t>
+          <t>054-8001447</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1380,7 +1380,7 @@
       <c r="H18" s="7" t="inlineStr"/>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בנתיבות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בקרית גת. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -1401,12 +1401,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>סנדרה קליניק</t>
+          <t>Svetlana Telerman קוסמטיקה אסתטית</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>ספיר</t>
+          <t>שדרות</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>050-6594249</t>
+          <t>052-3495811</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1424,10 +1424,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>קוסמטיקה אסתטית</t>
+        </is>
+      </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בספיר. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בשדרות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -1448,22 +1452,22 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>חורי הסרת שיער בלייזר</t>
+          <t>יעקב לייזר</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>ערד</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>050-9039052</t>
+          <t>052-5378645</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1471,10 +1475,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בערד. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -1495,22 +1503,22 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>פלאש לייזר Flash Laser</t>
+          <t>איזי לייזרס הסרת שיער</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>קרית גת</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>054-8001447</t>
+          <t>054-7618880</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1518,10 +1526,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער בלייזר</t>
+        </is>
+      </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בקרית גת. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
@@ -1542,22 +1554,22 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Svetlana Telerman קוסמטיקה אסתטית</t>
+          <t>מאסטרו לייזר לשיער וקעקועים</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>שדרות</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>דרום</t>
+          <t>ירושלים</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>052-3495811</t>
+          <t>054-4408964</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1567,12 +1579,12 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>קוסמטיקה אסתטית</t>
+          <t>לייזר לשיער ולהסרת קעקועים</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בשדרות. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -1593,7 +1605,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>יעקב לייזר</t>
+          <t>קליר אסטטיק</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1608,7 +1620,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>052-5378645</t>
+          <t>052-6609305</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1616,11 +1628,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
+      <c r="H23" s="7" t="inlineStr"/>
       <c r="I23" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -1644,7 +1652,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>איזי לייזרס הסרת שיער</t>
+          <t>rebecca לייזר וטיפולי RS</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1659,7 +1667,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>054-7618880</t>
+          <t>052-5921866</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1669,7 +1677,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>הסרת שיער בלייזר</t>
+          <t>לייזר וטיפולי RS</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -1695,7 +1703,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>מאסטרו לייזר לשיער וקעקועים</t>
+          <t>חיבה חזן קוסמטיקה</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1710,7 +1718,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>054-4408964</t>
+          <t>052-5482283</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1718,11 +1726,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>לייזר לשיער ולהסרת קעקועים</t>
-        </is>
-      </c>
+      <c r="H25" s="7" t="inlineStr"/>
       <c r="I25" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -1746,7 +1750,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>קליר אסטטיק</t>
+          <t>טטיאנה בולטקסוב</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1761,7 +1765,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>052-6609305</t>
+          <t>054-6903900</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1793,7 +1797,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>rebecca לייזר וטיפולי RS</t>
+          <t>רונית הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1808,7 +1812,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>052-5921866</t>
+          <t>054-3181660</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -1816,11 +1820,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>לייזר וטיפולי RS</t>
-        </is>
-      </c>
+      <c r="H27" s="7" t="inlineStr"/>
       <c r="I27" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>חיבה חזן קוסמטיקה</t>
+          <t>אור לייזר</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>052-5482283</t>
+          <t>052-5556107</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>טטיאנה בולטקסוב</t>
+          <t>אתי אשכנזי - המכון לקוסמטיקה מתקדמת</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>054-6903900</t>
+          <t>050-8684392</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -1938,22 +1938,22 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>רונית הסרת שיער בלייזר</t>
+          <t>מאסטר לייזר</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
+          <t>מעלה אדומים</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
           <t>ירושלים</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>054-3181660</t>
+          <t>054-2104112</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -1961,10 +1961,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr"/>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך במעלה אדומים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -1985,22 +1989,22 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>אור לייזר</t>
+          <t>עדן הסרת שיער</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>אורנית</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>052-5556107</t>
+          <t>050-3079554</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2011,7 +2015,7 @@
       <c r="H31" s="7" t="inlineStr"/>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך באורנית. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
@@ -2032,22 +2036,22 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>אתי אשכנזי - המכון לקוסמטיקה מתקדמת</t>
+          <t>מירב שילוני קוסמטיקה</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>אלעד</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>050-8684392</t>
+          <t>052-5556856</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -2055,10 +2059,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr"/>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>קוסמטיקה</t>
+        </is>
+      </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך באלעד. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -2079,22 +2087,22 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>מאסטר לייזר</t>
+          <t>שושי רווח קוסמטיקאית רפואית</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>מעלה אדומים</t>
+          <t>בית דגן</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>ירושלים</t>
+          <t>מרכז</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>054-2104112</t>
+          <t>052-2551019</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2104,12 +2112,12 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>מכון לייזר</t>
+          <t>קוסמטיקאית רפואית</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך במעלה אדומים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבית דגן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
@@ -2130,12 +2138,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>עדן הסרת שיער</t>
+          <t>Skin Flow by Rita Laser</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>אורנית</t>
+          <t>בני ברק</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2145,7 +2153,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>050-3079554</t>
+          <t>054-6909286</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2153,10 +2161,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך באורנית. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -2177,12 +2189,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>מירב שילוני קוסמטיקה</t>
+          <t>LAKOR הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>אלעד</t>
+          <t>בני ברק</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2192,7 +2204,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>052-5556856</t>
+          <t>053-3082606</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2202,12 +2214,12 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>קוסמטיקה</t>
+          <t>הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך באלעד. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J35" s="8" t="inlineStr">
@@ -2228,12 +2240,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>שושי רווח קוסמטיקאית רפואית</t>
+          <t>קליניק ארט - לגברים בלבד</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>בית דגן</t>
+          <t>בני ברק</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2243,7 +2255,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>052-2551019</t>
+          <t>054-7180190</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -2253,12 +2265,12 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>קוסמטיקאית רפואית</t>
+          <t>מכון לגברים בלבד</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבית דגן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -2279,7 +2291,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Skin Flow by Rita Laser</t>
+          <t>איזי לייזרס</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2294,7 +2306,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>054-6909286</t>
+          <t>054-5488969</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -2302,11 +2314,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
+      <c r="H37" s="7" t="inlineStr"/>
       <c r="I37" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -2330,12 +2338,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>LAKOR הסרת שיער בלייזר</t>
+          <t>אייקון אסטטיקס לייזר</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>בני ברק</t>
+          <t>ברקת</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -2345,7 +2353,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>053-3082606</t>
+          <t>054-9200681</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
@@ -2355,12 +2363,12 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>הסרת שיער בלייזר</t>
+          <t>אסתטיקה ולייזר</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בברקת. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -2381,12 +2389,12 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>קליניק ארט - לגברים בלבד</t>
+          <t>אלקיים יפעת</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>בני ברק</t>
+          <t>גבעתיים</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -2396,7 +2404,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>054-7180190</t>
+          <t>054-4268540</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -2404,14 +2412,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>מכון לגברים בלבד</t>
-        </is>
-      </c>
+      <c r="H39" s="7" t="inlineStr"/>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בגבעתיים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
@@ -2432,12 +2436,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>איזי לייזרס</t>
+          <t>אורין</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>בני ברק</t>
+          <t>גני תקווה</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2447,7 +2451,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>054-5488969</t>
+          <t>052-5787594</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -2458,7 +2462,7 @@
       <c r="H40" s="7" t="inlineStr"/>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבני ברק. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בגני תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -2479,12 +2483,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>אייקון אסטטיקס לייזר</t>
+          <t>חופית קוסמטיקה</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>ברקת</t>
+          <t>חולון</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2494,7 +2498,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>054-9200681</t>
+          <t>054-2186634</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
@@ -2504,12 +2508,12 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>אסתטיקה ולייזר</t>
+          <t>קוסמטיקה</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בברקת. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J41" s="8" t="inlineStr">
@@ -2530,12 +2534,12 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>אלקיים יפעת</t>
+          <t>קוסמטיק דניאל</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>גבעתיים</t>
+          <t>חולון</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -2545,7 +2549,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>054-4268540</t>
+          <t>050-6379038</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -2553,10 +2557,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>קוסמטיקה</t>
+        </is>
+      </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בגבעתיים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J42" s="8" t="inlineStr">
@@ -2577,12 +2585,12 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>אורין</t>
+          <t>חני שלמה הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>גני תקווה</t>
+          <t>חולון</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -2592,7 +2600,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>052-5787594</t>
+          <t>053-3916281</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -2600,10 +2608,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H43" s="7" t="inlineStr"/>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער בלייזר</t>
+        </is>
+      </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בגני תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J43" s="8" t="inlineStr">
@@ -2624,7 +2636,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>חופית קוסמטיקה</t>
+          <t>svetosh cosmetics</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2639,7 +2651,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>054-2186634</t>
+          <t>054-7508930</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -2675,7 +2687,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>קוסמטיק דניאל</t>
+          <t>מיכל בן דוד אפילציה</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -2690,7 +2702,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>050-6379038</t>
+          <t>050-8454658</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2698,11 +2710,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
-        <is>
-          <t>קוסמטיקה</t>
-        </is>
-      </c>
+      <c r="H45" s="7" t="inlineStr"/>
       <c r="I45" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -2726,7 +2734,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>חני שלמה הסרת שיער בלייזר</t>
+          <t>ליאורה לוי יחיאל אפילציה לנשים</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -2741,7 +2749,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>053-3916281</t>
+          <t>052-5757351</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2749,11 +2757,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער בלייזר</t>
-        </is>
-      </c>
+      <c r="H46" s="7" t="inlineStr"/>
       <c r="I46" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -2777,12 +2781,12 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>svetosh cosmetics</t>
+          <t>לירז קקון</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>חולון</t>
+          <t>יהוד</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -2792,7 +2796,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>054-7508930</t>
+          <t>054-7328238</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -2800,14 +2804,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>קוסמטיקה</t>
-        </is>
-      </c>
+      <c r="H47" s="7" t="inlineStr"/>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך ביהוד. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>מיכל בן דוד אפילציה</t>
+          <t>קרין קוסמטיקס</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>חולון</t>
+          <t>פתח תקווה</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>050-8454658</t>
+          <t>054-2844444</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
@@ -2851,10 +2851,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr"/>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>קוסמטיקה</t>
+        </is>
+      </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בפתח תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -2875,12 +2879,12 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>ליאורה לוי יחיאל אפילציה לנשים</t>
+          <t>קרן רונן הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>חולון</t>
+          <t>פתח תקווה</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -2890,7 +2894,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>052-5757351</t>
+          <t>050-4593281</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -2898,10 +2902,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr"/>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער בלייזר</t>
+        </is>
+      </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בחולון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בפתח תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J49" s="8" t="inlineStr">
@@ -2922,12 +2930,12 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>לירז קקון</t>
+          <t>קים סטרוגץ' - אפילציה</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>יהוד</t>
+          <t>פתח תקווה</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -2937,7 +2945,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>054-7328238</t>
+          <t>053-2203822</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
@@ -2945,10 +2953,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr"/>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער לצמיתות באפילציה</t>
+        </is>
+      </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך ביהוד. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בפתח תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -2969,7 +2981,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>קרין קוסמטיקס</t>
+          <t>חגית הסרת שיער</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2984,7 +2996,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>054-2844444</t>
+          <t>052-5789438</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -2994,7 +3006,7 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>קוסמטיקה</t>
+          <t>הסרת שיער</t>
         </is>
       </c>
       <c r="I51" s="7" t="inlineStr">
@@ -3020,12 +3032,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>קרן רונן הסרת שיער בלייזר</t>
+          <t>זיוה מלכה קוסמטיקאית פרא-רפואית</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>פתח תקווה</t>
+          <t>קרית אונו</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
@@ -3035,7 +3047,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>050-4593281</t>
+          <t>050-6707037</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -3045,12 +3057,12 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>הסרת שיער בלייזר</t>
+          <t>קוסמטיקאית פרא-רפואית</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בפתח תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בקרית אונו. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -3071,12 +3083,12 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>קים סטרוגץ' - אפילציה</t>
+          <t>איריס הסרת שיער</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>פתח תקווה</t>
+          <t>קרית אונו</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -3086,7 +3098,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>053-2203822</t>
+          <t>050-4567690</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -3096,12 +3108,12 @@
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>הסרת שיער לצמיתות באפילציה</t>
+          <t>הסרת שיער</t>
         </is>
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בפתח תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בקרית אונו. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
@@ -3122,12 +3134,12 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>חגית הסרת שיער</t>
+          <t>אור אסטטיק</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>פתח תקווה</t>
+          <t>ראש העין</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -3137,7 +3149,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>052-5789438</t>
+          <t>052-8736622</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -3147,12 +3159,12 @@
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>הסרת שיער</t>
+          <t>אסתטיקה</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בפתח תקווה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בראש העין. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -3173,12 +3185,12 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>זיוה מלכה קוסמטיקאית פרא-רפואית</t>
+          <t>טוני מכון לייזר</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>קרית אונו</t>
+          <t>ראש העין</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -3188,7 +3200,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>050-6707037</t>
+          <t>053-3007781</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -3198,12 +3210,12 @@
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>קוסמטיקאית פרא-רפואית</t>
+          <t>מכון לייזר</t>
         </is>
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בקרית אונו. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בראש העין. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J55" s="8" t="inlineStr">
@@ -3224,12 +3236,12 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>איריס הסרת שיער</t>
+          <t>רומיס קליניק</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>קרית אונו</t>
+          <t>ראשון לציון</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -3239,7 +3251,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>050-4567690</t>
+          <t>054-2424231</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -3249,12 +3261,12 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>הסרת שיער</t>
+          <t>קליניקה</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בקרית אונו. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -3275,12 +3287,12 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>אור אסטטיק</t>
+          <t>מסירים - הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>ראש העין</t>
+          <t>ראשון לציון</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -3290,7 +3302,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>052-8736622</t>
+          <t>054-3332825</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -3298,14 +3310,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
-        <is>
-          <t>אסתטיקה</t>
-        </is>
-      </c>
+      <c r="H57" s="7" t="inlineStr"/>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בראש העין. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
@@ -3326,12 +3334,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>טוני מכון לייזר</t>
+          <t>לירז מאיו הסרת שיער</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>ראש העין</t>
+          <t>ראשון לציון</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -3341,7 +3349,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>053-3007781</t>
+          <t>050-7114452</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -3349,14 +3357,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
+      <c r="H58" s="7" t="inlineStr"/>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בראש העין. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -3377,7 +3381,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>רומיס קליניק</t>
+          <t>NK Clinic הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -3392,7 +3396,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>054-2424231</t>
+          <t>052-7497762</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -3400,11 +3404,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
-        <is>
-          <t>קליניקה</t>
-        </is>
-      </c>
+      <c r="H59" s="7" t="inlineStr"/>
       <c r="I59" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -3428,12 +3428,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>מסירים - הסרת שיער בלייזר</t>
+          <t>ענבל ויס הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>ראשון לציון</t>
+          <t>רמת גן</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>054-3332825</t>
+          <t>050-9383038</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
@@ -3451,10 +3451,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr"/>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>הסרת שיער בלייזר</t>
+        </is>
+      </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -3475,12 +3479,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>לירז מאיו הסרת שיער</t>
+          <t>דליה אפילציה</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>ראשון לציון</t>
+          <t>רמת גן</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
@@ -3490,7 +3494,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>050-7114452</t>
+          <t>052-3643757</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -3501,7 +3505,7 @@
       <c r="H61" s="7" t="inlineStr"/>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J61" s="8" t="inlineStr">
@@ -3522,12 +3526,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>NK Clinic הסרת שיער בלייזר</t>
+          <t>רות קוסמטיקס</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>ראשון לציון</t>
+          <t>רמת גן</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -3537,7 +3541,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>052-7497762</t>
+          <t>052-7499555</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -3548,7 +3552,7 @@
       <c r="H62" s="7" t="inlineStr"/>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בראשון לציון. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
@@ -3569,7 +3573,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>ענבל ויס הסרת שיער בלייזר</t>
+          <t>אפילציה גילי</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -3584,7 +3588,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>050-9383038</t>
+          <t>052-2451863</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">
@@ -3592,11 +3596,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H63" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער בלייזר</t>
-        </is>
-      </c>
+      <c r="H63" s="7" t="inlineStr"/>
       <c r="I63" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -3620,12 +3620,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>דליה אפילציה</t>
+          <t>לירז קוסמטיקה</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>רמת גן</t>
+          <t>תל אביב</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>052-3643757</t>
+          <t>052-6865368</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -3643,10 +3643,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr"/>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>קוסמטיקה</t>
+        </is>
+      </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
@@ -3667,12 +3671,12 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>רות קוסמטיקס</t>
+          <t>קרן לייזר</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>רמת גן</t>
+          <t>תל אביב</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
@@ -3682,7 +3686,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>052-7499555</t>
+          <t>052-4841470</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -3690,10 +3694,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H65" s="7" t="inlineStr"/>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J65" s="8" t="inlineStr">
@@ -3714,12 +3722,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>אפילציה גילי</t>
+          <t>Rk laser</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>רמת גן</t>
+          <t>תל אביב</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -3729,7 +3737,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>052-2451863</t>
+          <t>054-6234954</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
@@ -3737,10 +3745,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr"/>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך ברמת גן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J66" s="8" t="inlineStr">
@@ -3761,7 +3773,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>לירז קוסמטיקה</t>
+          <t>אולסטרס לייזר</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -3776,7 +3788,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>052-6865368</t>
+          <t>053-5540319</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -3786,7 +3798,7 @@
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>קוסמטיקה</t>
+          <t>מכון לייזר</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -3812,7 +3824,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>קרן לייזר</t>
+          <t>Laser King</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -3827,7 +3839,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>052-4841470</t>
+          <t>053-7147539</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -3863,7 +3875,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Rk laser</t>
+          <t>טכנו קוסמטיקס</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -3878,7 +3890,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>054-6234954</t>
+          <t>050-3369697</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr">
@@ -3886,11 +3898,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H69" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
+      <c r="H69" s="7" t="inlineStr"/>
       <c r="I69" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -3914,7 +3922,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>אולסטרס לייזר</t>
+          <t>YClinique</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -3929,7 +3937,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>053-5540319</t>
+          <t>050-9082672</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
@@ -3937,11 +3945,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
+      <c r="H70" s="7" t="inlineStr"/>
       <c r="I70" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -3965,7 +3969,7 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Laser King</t>
+          <t>נו בודי הייר</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -3980,7 +3984,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>053-7147539</t>
+          <t>054-4449661</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr">
@@ -3988,11 +3992,7 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
+      <c r="H71" s="7" t="inlineStr"/>
       <c r="I71" s="7" t="inlineStr">
         <is>
           <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>טכנו קוסמטיקס</t>
+          <t>אסיפרה</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>050-3369697</t>
+          <t>054-6855723</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>YClinique</t>
+          <t>אורנוס לייזר</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>050-9082672</t>
+          <t>050-7157155</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>נו בודי הייר</t>
+          <t>נטלי שוסטר</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>054-4449661</t>
+          <t>050-9110999</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -4157,22 +4157,22 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>אסיפרה</t>
+          <t>ארמון היופי</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>תל אביב</t>
+          <t>בית ג'ן</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>054-6855723</t>
+          <t>054-3101646</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -4183,7 +4183,7 @@
       <c r="H75" s="7" t="inlineStr"/>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבית ג'ן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J75" s="8" t="inlineStr">
@@ -4204,22 +4204,22 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>אורנוס לייזר</t>
+          <t>אפרת יופי של מקום</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>תל אביב</t>
+          <t>בית לחם הגלילית</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>050-7157155</t>
+          <t>052-2852208</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
@@ -4230,7 +4230,7 @@
       <c r="H76" s="7" t="inlineStr"/>
       <c r="I76" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בבית לחם הגלילית. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J76" s="8" t="inlineStr">
@@ -4251,22 +4251,22 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>נטלי שוסטר</t>
+          <t>LightCare</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>תל אביב</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>מרכז</t>
+          <t>צפון</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>050-9110999</t>
+          <t>054-3303411</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
@@ -4274,10 +4274,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H77" s="7" t="inlineStr"/>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>שני סניפים: חיפה ויקנעם</t>
+        </is>
+      </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בתל אביב. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J77" s="8" t="inlineStr">
@@ -4298,12 +4302,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>ארמון היופי</t>
+          <t>בסנת ביוטי קליניק</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>בית ג'ן</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -4313,7 +4317,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>054-3101646</t>
+          <t>054-3117484</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr">
@@ -4321,10 +4325,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H78" s="7" t="inlineStr"/>
+      <c r="H78" s="7" t="inlineStr">
+        <is>
+          <t>שד׳ בן גוריון</t>
+        </is>
+      </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבית ג'ן. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J78" s="8" t="inlineStr">
@@ -4345,12 +4353,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>אפרת יופי של מקום</t>
+          <t>סקיניק לייזר</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>בית לחם הגלילית</t>
+          <t>חיפה</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -4360,7 +4368,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>052-2852208</t>
+          <t>052-5552191</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
@@ -4368,10 +4376,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H79" s="7" t="inlineStr"/>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בבית לחם הגלילית. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J79" s="8" t="inlineStr">
@@ -4392,12 +4404,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>LightCare</t>
+          <t>זברה zebra cosmetics</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>חיפה</t>
+          <t>טירת כרמל</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -4407,7 +4419,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>054-3303411</t>
+          <t>058-7011140</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr">
@@ -4415,14 +4427,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H80" s="7" t="inlineStr">
-        <is>
-          <t>שני סניפים: חיפה ויקנעם</t>
-        </is>
-      </c>
+      <c r="H80" s="7" t="inlineStr"/>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בטירת כרמל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J80" s="8" t="inlineStr">
@@ -4443,12 +4451,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>בסנת ביוטי קליניק</t>
+          <t>רונית איכילוב הסרת שיער</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>חיפה</t>
+          <t>כרמיאל</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -4458,7 +4466,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>054-3117484</t>
+          <t>054-3305141</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
@@ -4468,12 +4476,12 @@
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>שד׳ בן גוריון</t>
+          <t>הסרת שיער</t>
         </is>
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בכרמיאל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J81" s="8" t="inlineStr">
@@ -4494,12 +4502,12 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>סקיניק לייזר</t>
+          <t>אן קליניק</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>חיפה</t>
+          <t>כרמיאל</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -4509,7 +4517,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>052-5552191</t>
+          <t>054-2128090</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
@@ -4519,12 +4527,12 @@
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>מכון לייזר</t>
+          <t>בקניון כיכר העיר</t>
         </is>
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בכרמיאל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J82" s="8" t="inlineStr">
@@ -4545,12 +4553,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>זברה zebra cosmetics</t>
+          <t>הפינוק בלוק</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>טירת כרמל</t>
+          <t>כרמיאל</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -4560,7 +4568,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>058-7011140</t>
+          <t>050-7375638</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
@@ -4571,7 +4579,7 @@
       <c r="H83" s="7" t="inlineStr"/>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בטירת כרמל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בכרמיאל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J83" s="8" t="inlineStr">
@@ -4592,12 +4600,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>רונית איכילוב הסרת שיער</t>
+          <t>משי הסרת שיער</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>כרמיאל</t>
+          <t>לוטם</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -4607,7 +4615,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>054-3305141</t>
+          <t>050-5661398</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
@@ -4615,14 +4623,10 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער</t>
-        </is>
-      </c>
+      <c r="H84" s="7" t="inlineStr"/>
       <c r="I84" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בכרמיאל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בלוטם. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J84" s="8" t="inlineStr">
@@ -4643,12 +4647,12 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>אן קליניק</t>
+          <t>רעות הדר הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>כרמיאל</t>
+          <t>מעלות-תרשיחא</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -4658,7 +4662,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>054-2128090</t>
+          <t>052-4394616</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -4668,12 +4672,12 @@
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>בקניון כיכר העיר</t>
+          <t>הסרת שיער בלייזר</t>
         </is>
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בכרמיאל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך במעלות-תרשיחא. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J85" s="8" t="inlineStr">
@@ -4694,12 +4698,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>הפינוק בלוק</t>
+          <t>נטלי לייזר</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>כרמיאל</t>
+          <t>נהריה</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
@@ -4709,7 +4713,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>050-7375638</t>
+          <t>053-3309281</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr">
@@ -4717,10 +4721,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H86" s="7" t="inlineStr"/>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I86" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בכרמיאל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בנהריה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
@@ -4741,12 +4749,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>משי הסרת שיער</t>
+          <t>דרים לייזר</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>לוטם</t>
+          <t>קרית ים</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -4756,7 +4764,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>050-5661398</t>
+          <t>053-3894054</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
@@ -4764,10 +4772,14 @@
           <t>וואטסאפ</t>
         </is>
       </c>
-      <c r="H87" s="7" t="inlineStr"/>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>מכון לייזר</t>
+        </is>
+      </c>
       <c r="I87" s="7" t="inlineStr">
         <is>
-          <t>ראיתי את המכון שלך בלוטם. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
+          <t>ראיתי את המכון שלך בקרית ים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
         </is>
       </c>
       <c r="J87" s="8" t="inlineStr">
@@ -4777,706 +4789,186 @@
       </c>
       <c r="K87" s="9" t="inlineStr"/>
     </row>
-    <row r="88">
-      <c r="A88" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>ב</t>
-        </is>
-      </c>
-      <c r="C88" s="3" t="inlineStr">
-        <is>
-          <t>רעות הדר הסרת שיער בלייזר</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>מעלות-תרשיחא</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr">
-        <is>
-          <t>052-4394616</t>
-        </is>
-      </c>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>וואטסאפ</t>
-        </is>
-      </c>
-      <c r="H88" s="7" t="inlineStr">
-        <is>
-          <t>הסרת שיער בלייזר</t>
-        </is>
-      </c>
-      <c r="I88" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך במעלות-תרשיחא. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J88" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K88" s="9" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>ב</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t>נטלי לייזר</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>נהריה</t>
-        </is>
-      </c>
-      <c r="E89" s="4" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="F89" s="5" t="inlineStr">
-        <is>
-          <t>053-3309281</t>
-        </is>
-      </c>
-      <c r="G89" s="6" t="inlineStr">
-        <is>
-          <t>וואטסאפ</t>
-        </is>
-      </c>
-      <c r="H89" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
-      <c r="I89" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בנהריה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J89" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K89" s="9" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>ב</t>
-        </is>
-      </c>
-      <c r="C90" s="3" t="inlineStr">
-        <is>
-          <t>דרים לייזר</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>קרית ים</t>
-        </is>
-      </c>
-      <c r="E90" s="4" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
-          <t>053-3894054</t>
-        </is>
-      </c>
-      <c r="G90" s="6" t="inlineStr">
-        <is>
-          <t>וואטסאפ</t>
-        </is>
-      </c>
-      <c r="H90" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
-      <c r="I90" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בקרית ים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J90" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K90" s="9" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C91" s="3" t="inlineStr">
-        <is>
-          <t>יופי וטבע זוהרה</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>קרית גת</t>
-        </is>
-      </c>
-      <c r="E91" s="4" t="inlineStr">
-        <is>
-          <t>דרום</t>
-        </is>
-      </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>08-6810707</t>
-        </is>
-      </c>
-      <c r="G91" s="6" t="inlineStr"/>
-      <c r="H91" s="7" t="inlineStr">
-        <is>
-          <t>"מכון הקוסמטיקה והלייזר הוותיק בדרום"</t>
-        </is>
-      </c>
-      <c r="I91" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בקרית גת. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J91" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K91" s="9" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="inlineStr">
-        <is>
-          <t>לייזעור</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>02-5655605</t>
-        </is>
-      </c>
-      <c r="G92" s="6" t="inlineStr"/>
-      <c r="H92" s="7" t="inlineStr"/>
-      <c r="I92" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J92" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K92" s="9" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="inlineStr">
-        <is>
-          <t>המכון ללייזר - ד"ר מוסיה</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
-          <t>02-5879596</t>
-        </is>
-      </c>
-      <c r="G93" s="6" t="inlineStr"/>
-      <c r="H93" s="7" t="inlineStr"/>
-      <c r="I93" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J93" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K93" s="9" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C94" s="3" t="inlineStr">
-        <is>
-          <t>סיגל כנעני - אפילציה</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="E94" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
-          <t>02-6763663</t>
-        </is>
-      </c>
-      <c r="G94" s="6" t="inlineStr"/>
-      <c r="H94" s="7" t="inlineStr"/>
-      <c r="I94" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J94" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K94" s="9" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C95" s="3" t="inlineStr">
-        <is>
-          <t>bellissima אסטטיקה מתקדמת</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>ירושלים</t>
-        </is>
-      </c>
-      <c r="F95" s="5" t="inlineStr">
-        <is>
-          <t>02-6504624</t>
-        </is>
-      </c>
-      <c r="G95" s="6" t="inlineStr"/>
-      <c r="H95" s="7" t="inlineStr"/>
-      <c r="I95" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בירושלים. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J95" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K95" s="9" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t>המרכז להרחקת שיער אקטיב לייט</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>אזור</t>
-        </is>
-      </c>
-      <c r="E96" s="4" t="inlineStr">
-        <is>
-          <t>מרכז</t>
-        </is>
-      </c>
-      <c r="F96" s="5" t="inlineStr">
-        <is>
-          <t>03-5560454</t>
-        </is>
-      </c>
-      <c r="G96" s="6" t="inlineStr"/>
-      <c r="H96" s="7" t="inlineStr"/>
-      <c r="I96" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך באזור. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J96" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K96" s="9" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>לייזר הכרמל</t>
-        </is>
-      </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>דאלית אל-כרמל</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="F97" s="5" t="inlineStr">
-        <is>
-          <t>04-8396811</t>
-        </is>
-      </c>
-      <c r="G97" s="6" t="inlineStr"/>
-      <c r="H97" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
-      <c r="I97" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בדאלית אל-כרמל. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J97" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K97" s="9" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>ג</t>
-        </is>
-      </c>
-      <c r="C98" s="3" t="inlineStr">
-        <is>
-          <t>מדיקל אם - מכון לייזר</t>
-        </is>
-      </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>חיפה</t>
-        </is>
-      </c>
-      <c r="E98" s="4" t="inlineStr">
-        <is>
-          <t>צפון</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>04-6217007</t>
-        </is>
-      </c>
-      <c r="G98" s="6" t="inlineStr"/>
-      <c r="H98" s="7" t="inlineStr">
-        <is>
-          <t>מכון לייזר</t>
-        </is>
-      </c>
-      <c r="I98" s="7" t="inlineStr">
-        <is>
-          <t>ראיתי את המכון שלך בחיפה. שאלה קצרה: כשליד נכנס ואת באמצע טיפול, תוך כמה זמן את חוזרת אליה?</t>
-        </is>
-      </c>
-      <c r="J98" s="8" t="inlineStr">
-        <is>
-          <t>לא התקשרתי</t>
-        </is>
-      </c>
-      <c r="K98" s="9" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K98"/>
+  <autoFilter ref="A1:K87"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"לא התקשרתי,לא ענתה,לחזור אליה,נקבע דמו,לא מעוניינת,נסגר!"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F97" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId172"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>